<commit_message>
Menus: remove prices, charges and UPI pay
Prices changed faster than the cards could be re-typed. Night canteen and
tuck shop menus now list dishes only: no item prices, no room-service or
delivery fees, no basket totals, and no UPI pay block or shop QRs. The
basket and WhatsApp message carry names and quantities; the tuck "Deliver
to" picker stays, without fees. Order history no longer shows or exports
a basket total.

The build scripts, templates and source workbooks drop the Price, room
service, fee and UPI columns (workbook backups are *.before-2026-10-29.xlsx
in rollcall-resources). Tuck Info's "Delivery (Rs)" becomes "Delivers".
test/logic.mjs fails if a price returns to the menu data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Night Mess Menu.template.xlsx
+++ b/templates/Night Mess Menu.template.xlsx
@@ -429,14 +429,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,11 +459,6 @@
           <t>Hours</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Room service (Rs)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -487,9 +481,6 @@
           <t>11:00 PM - 4:00 AM</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -511,9 +502,6 @@
         <is>
           <t>11:00 PM - 4:00 AM</t>
         </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -527,13 +515,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,11 +536,6 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
           <t>Diet</t>
         </is>
       </c>
@@ -569,10 +551,7 @@
           <t>Veg Roll</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>veg</t>
         </is>
@@ -589,10 +568,7 @@
           <t>Egg Roll</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>egg</t>
         </is>
@@ -609,10 +585,7 @@
           <t>Chicken Roll</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>non-veg</t>
         </is>
@@ -629,10 +602,7 @@
           <t>Veg Steam Momo</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>veg</t>
         </is>
@@ -649,10 +619,7 @@
           <t>Chicken Steam Momo</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>non-veg</t>
         </is>
@@ -670,11 +637,6 @@
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>22/25</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>veg</t>
         </is>
@@ -691,13 +653,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -713,11 +674,6 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
           <t>Diet</t>
         </is>
       </c>
@@ -733,10 +689,7 @@
           <t>Veg Roll</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>veg</t>
         </is>
@@ -753,10 +706,7 @@
           <t>Egg Roll</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>egg</t>
         </is>
@@ -773,10 +723,7 @@
           <t>Chicken Roll</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>non-veg</t>
         </is>
@@ -793,10 +740,7 @@
           <t>Veg Steam Momo</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>veg</t>
         </is>
@@ -813,10 +757,7 @@
           <t>Chicken Steam Momo</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>non-veg</t>
         </is>
@@ -834,11 +775,6 @@
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>22/25</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>veg</t>
         </is>

</xml_diff>